<commit_message>
Copilot-ready xlsx: data rows as Excel table ExecutionReport; inspector updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4wyHvWAGZBDCUAjTzmt7H
</commit_message>
<xml_diff>
--- a/copilot-kit/fy26_q3_execution_report.xlsx
+++ b/copilot-kit/fy26_q3_execution_report.xlsx
@@ -341,6 +341,27 @@
 </styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ExecutionReport" displayName="ExecutionReport" ref="A5:L30" totalsRowShown="0">
+  <autoFilter ref="A5:L30"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="Code"/>
+    <tableColumn id="2" name="Program / activity"/>
+    <tableColumn id="3" name="FY26 annual plan"/>
+    <tableColumn id="4" name="Q3 obligation plan"/>
+    <tableColumn id="5" name="Obligations"/>
+    <tableColumn id="6" name="Obligation variance"/>
+    <tableColumn id="7" name="Obligation variance %"/>
+    <tableColumn id="8" name="Q3 expenditure plan"/>
+    <tableColumn id="9" name="Expenditures"/>
+    <tableColumn id="10" name="Expenditure variance"/>
+    <tableColumn id="11" name="Expenditure variance %"/>
+    <tableColumn id="12" name="Remarks"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
@@ -1472,5 +1493,8 @@
   </sheetData>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Relatable example: SYN-107/109 without remarks (AI must infer or ask), Demo 2 as a program-office data call with audit close, approved-systems line
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4wyHvWAGZBDCUAjTzmt7H
</commit_message>
<xml_diff>
--- a/copilot-kit/fy26_q3_execution_report.xlsx
+++ b/copilot-kit/fy26_q3_execution_report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
   <si>
     <t xml:space="preserve">FY26 Q3 Execution Report — Operation and Maintenance (O&amp;M)</t>
   </si>
@@ -113,9 +113,6 @@
     <t xml:space="preserve">End-User Device Refresh</t>
   </si>
   <si>
-    <t xml:space="preserve">One-time purchase of 1,150 replacement workstations (end of life), approved by resource board 2 Jun; unit cost below expense/investment threshold.</t>
-  </si>
-  <si>
     <t xml:space="preserve">SYN-108</t>
   </si>
   <si>
@@ -129,9 +126,6 @@
   </si>
   <si>
     <t xml:space="preserve">Mission Support Services</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Task order obligated on schedule; contractor invoices for Apr–Jun not yet received.</t>
   </si>
   <si>
     <t xml:space="preserve">SYN-110</t>
@@ -721,16 +715,13 @@
         <f>IF(H12=0,0,J12/H12)</f>
         <v>0.28125</v>
       </c>
-      <c r="L12" s="6" t="s">
-        <v>33</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="0" t="s">
         <v>34</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>35</v>
       </c>
       <c r="C13" s="4">
         <v>3800</v>
@@ -764,15 +755,15 @@
         <v>0.005</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="0" t="s">
         <v>37</v>
-      </c>
-      <c r="B14" s="0" t="s">
-        <v>38</v>
       </c>
       <c r="C14" s="4">
         <v>7200</v>
@@ -805,16 +796,13 @@
         <f>IF(H14=0,0,J14/H14)</f>
         <v>-0.6341463414634146</v>
       </c>
-      <c r="L14" s="6" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C15" s="4">
         <v>5600</v>
@@ -850,10 +838,10 @@
     </row>
     <row r="16">
       <c r="A16" s="0" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C16" s="4">
         <v>1600</v>
@@ -889,10 +877,10 @@
     </row>
     <row r="17">
       <c r="A17" s="0" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C17" s="4">
         <v>600</v>
@@ -928,10 +916,10 @@
     </row>
     <row r="18">
       <c r="A18" s="0" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C18" s="4">
         <v>1200</v>
@@ -967,10 +955,10 @@
     </row>
     <row r="19">
       <c r="A19" s="0" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C19" s="4">
         <v>300</v>
@@ -1006,10 +994,10 @@
     </row>
     <row r="20">
       <c r="A20" s="0" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B20" s="0" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C20" s="4">
         <v>4000</v>
@@ -1045,10 +1033,10 @@
     </row>
     <row r="21">
       <c r="A21" s="0" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C21" s="4">
         <v>2400</v>
@@ -1084,10 +1072,10 @@
     </row>
     <row r="22">
       <c r="A22" s="0" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C22" s="4">
         <v>900</v>
@@ -1123,10 +1111,10 @@
     </row>
     <row r="23">
       <c r="A23" s="0" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C23" s="4">
         <v>2000</v>
@@ -1162,10 +1150,10 @@
     </row>
     <row r="24">
       <c r="A24" s="0" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B24" s="0" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C24" s="4">
         <v>3200</v>
@@ -1201,10 +1189,10 @@
     </row>
     <row r="25">
       <c r="A25" s="0" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B25" s="0" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C25" s="4">
         <v>4400</v>
@@ -1238,15 +1226,15 @@
         <v>-0.028</v>
       </c>
       <c r="L25" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="0" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C26" s="4">
         <v>1800</v>
@@ -1282,10 +1270,10 @@
     </row>
     <row r="27">
       <c r="A27" s="0" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C27" s="4">
         <v>2600</v>
@@ -1321,10 +1309,10 @@
     </row>
     <row r="28">
       <c r="A28" s="0" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C28" s="4">
         <v>500</v>
@@ -1360,10 +1348,10 @@
     </row>
     <row r="29">
       <c r="A29" s="0" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C29" s="4">
         <v>1400</v>
@@ -1399,10 +1387,10 @@
     </row>
     <row r="30">
       <c r="A30" s="0" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C30" s="4">
         <v>700</v>
@@ -1438,10 +1426,10 @@
     </row>
     <row r="31">
       <c r="A31" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C31" s="8">
         <f>SUM(C6:C30)</f>
@@ -1482,12 +1470,12 @@
     </row>
     <row r="33">
       <c r="A33" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>